<commit_message>
Akwizycja danych, lab 1: slajdy wstępu, instrukcja (wykres XY, dashboard krok po kroku), rozdzielone pola wyników
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/akwizycja-danych/lab-1/Lab_1_Pakowaczka01.xlsx
+++ b/akwizycja-danych/lab-1/Lab_1_Pakowaczka01.xlsx
@@ -18,10 +18,12 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="3">
+  <numFmts count="5">
     <numFmt numFmtId="164" formatCode="yyyy-mm-dd h:mm:ss"/>
     <numFmt numFmtId="165" formatCode="yyyy-mm-dd hh:mm:ss"/>
     <numFmt numFmtId="166" formatCode="0.0"/>
+    <numFmt numFmtId="167" formatCode="0.0%"/>
+    <numFmt numFmtId="168" formatCode="hh:mm:ss"/>
   </numFmts>
   <fonts count="3">
     <font>
@@ -83,7 +85,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="11">
+  <cellXfs count="16">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
@@ -91,14 +93,31 @@
     <xf numFmtId="165" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="166" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="2" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="3" fontId="0" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="1" fontId="0" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="166" fontId="0" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="167" fontId="0" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="2" fontId="0" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="168" fontId="0" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -477,6 +496,12 @@
     <col width="12" customWidth="1" min="6" max="6"/>
     <col width="14" customWidth="1" min="7" max="7"/>
     <col width="12" customWidth="1" min="8" max="8"/>
+    <col width="11" customWidth="1" min="9" max="9"/>
+    <col width="11" customWidth="1" min="10" max="10"/>
+    <col width="11" customWidth="1" min="11" max="11"/>
+    <col width="9" customWidth="1" min="12" max="12"/>
+    <col width="9" customWidth="1" min="13" max="13"/>
+    <col width="9" customWidth="1" min="14" max="14"/>
   </cols>
   <sheetData>
     <row r="1" ht="32" customHeight="1">
@@ -78008,530 +78033,657 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D31"/>
+  <dimension ref="A1:D39"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
-    <col width="58" customWidth="1" min="2" max="2"/>
+    <col width="52" customWidth="1" min="2" max="2"/>
     <col width="46" customWidth="1" min="3" max="3"/>
     <col width="9" customWidth="1" min="4" max="4"/>
   </cols>
   <sheetData>
-    <row r="1">
+    <row r="1" ht="24" customHeight="1">
       <c r="A1" s="5" t="inlineStr">
         <is>
+          <t>Zespół (1–2 osoby): imię i nazwisko</t>
+        </is>
+      </c>
+      <c r="C1" s="6" t="inlineStr"/>
+    </row>
+    <row r="3">
+      <c r="A3" s="7" t="inlineStr">
+        <is>
           <t>Nr</t>
         </is>
       </c>
-      <c r="B1" s="5" t="inlineStr">
+      <c r="B3" s="7" t="inlineStr">
         <is>
           <t>Pytanie</t>
         </is>
       </c>
-      <c r="C1" s="5" t="inlineStr">
+      <c r="C3" s="7" t="inlineStr">
         <is>
           <t>Wynik</t>
         </is>
       </c>
-      <c r="D1" s="5" t="inlineStr">
+      <c r="D3" s="7" t="inlineStr">
         <is>
           <t>Jedn.</t>
         </is>
       </c>
     </row>
-    <row r="2" ht="22" customHeight="1">
-      <c r="A2" s="6" t="inlineStr">
-        <is>
-          <t>Zespół (1–2 osoby): imię i nazwisko</t>
-        </is>
-      </c>
-      <c r="B2" s="7" t="inlineStr"/>
-    </row>
-    <row r="3">
-      <c r="A3" s="8" t="inlineStr">
+    <row r="4">
+      <c r="A4" s="5" t="inlineStr">
         <is>
           <t>Blok 1 — oględziny danych</t>
         </is>
       </c>
     </row>
-    <row r="4">
-      <c r="A4" s="9" t="inlineStr">
+    <row r="5">
+      <c r="A5" s="8" t="inlineStr">
         <is>
           <t>1a</t>
         </is>
       </c>
-      <c r="B4" s="9" t="inlineStr">
+      <c r="B5" s="8" t="inlineStr">
         <is>
           <t>Liczba rekordów w arkuszu Dane (bez nagłówka)</t>
         </is>
       </c>
-      <c r="C4" s="10" t="inlineStr"/>
-      <c r="D4" s="9" t="inlineStr">
+      <c r="C5" s="9" t="inlineStr"/>
+      <c r="D5" s="8" t="inlineStr">
         <is>
           <t>szt.</t>
         </is>
       </c>
     </row>
-    <row r="5">
-      <c r="A5" s="9" t="inlineStr">
+    <row r="6">
+      <c r="A6" s="8" t="inlineStr">
         <is>
           <t>1b</t>
         </is>
       </c>
-      <c r="B5" s="9" t="inlineStr">
+      <c r="B6" s="8" t="inlineStr">
         <is>
           <t>Co ile sekund zapisywane są rekordy?</t>
         </is>
       </c>
-      <c r="C5" s="10" t="inlineStr"/>
-      <c r="D5" s="9" t="inlineStr">
+      <c r="C6" s="10" t="inlineStr"/>
+      <c r="D6" s="8" t="inlineStr">
         <is>
           <t>s</t>
         </is>
       </c>
     </row>
-    <row r="6" ht="60" customHeight="1">
-      <c r="A6" s="9" t="inlineStr">
+    <row r="7" ht="60" customHeight="1">
+      <c r="A7" s="8" t="inlineStr">
         <is>
           <t>2</t>
         </is>
       </c>
-      <c r="B6" s="9" t="inlineStr">
+      <c r="B7" s="8" t="inlineStr">
         <is>
           <t>Podejrzane miejsca w danych: godzina + co widać (min. 3)</t>
         </is>
       </c>
-      <c r="C6" s="10" t="inlineStr"/>
-      <c r="D6" s="9" t="inlineStr">
+      <c r="C7" s="11" t="inlineStr"/>
+      <c r="D7" s="8" t="inlineStr">
         <is>
           <t>opis</t>
         </is>
       </c>
     </row>
-    <row r="7">
-      <c r="A7" s="8" t="inlineStr">
+    <row r="8">
+      <c r="A8" s="5" t="inlineStr">
         <is>
           <t>Blok 2 — czyszczenie danych</t>
         </is>
       </c>
     </row>
-    <row r="8">
-      <c r="A8" s="9" t="inlineStr">
+    <row r="9">
+      <c r="A9" s="8" t="inlineStr">
         <is>
           <t>3</t>
         </is>
       </c>
-      <c r="B8" s="9" t="inlineStr">
-        <is>
-          <t>Ile duplikatów usunięto? Ile rekordów zostało?</t>
-        </is>
-      </c>
-      <c r="C8" s="10" t="inlineStr"/>
-      <c r="D8" s="9" t="inlineStr">
+      <c r="B9" s="8" t="inlineStr">
+        <is>
+          <t>Ile duplikatów usunięto?</t>
+        </is>
+      </c>
+      <c r="C9" s="9" t="inlineStr"/>
+      <c r="D9" s="8" t="inlineStr">
         <is>
           <t>szt.</t>
         </is>
       </c>
     </row>
-    <row r="9">
-      <c r="A9" s="9" t="inlineStr">
+    <row r="10">
+      <c r="A10" s="8" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="B10" s="8" t="inlineStr">
+        <is>
+          <t>Ile rekordów zostało?</t>
+        </is>
+      </c>
+      <c r="C10" s="9" t="inlineStr"/>
+      <c r="D10" s="8" t="inlineStr">
+        <is>
+          <t>szt.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="8" t="inlineStr">
         <is>
           <t>4a</t>
         </is>
       </c>
-      <c r="B9" s="9" t="inlineStr">
+      <c r="B11" s="8" t="inlineStr">
         <is>
           <t>Średnia temperatura zgrzewu — przed usunięciem zer</t>
         </is>
       </c>
-      <c r="C9" s="10" t="inlineStr"/>
-      <c r="D9" s="9" t="inlineStr">
+      <c r="C11" s="12" t="inlineStr"/>
+      <c r="D11" s="8" t="inlineStr">
         <is>
           <t>°C</t>
         </is>
       </c>
     </row>
-    <row r="10">
-      <c r="A10" s="9" t="inlineStr">
+    <row r="12">
+      <c r="A12" s="8" t="inlineStr">
         <is>
           <t>4b</t>
         </is>
       </c>
-      <c r="B10" s="9" t="inlineStr">
+      <c r="B12" s="8" t="inlineStr">
         <is>
           <t>Średnia temperatura zgrzewu — po usunięciu zer</t>
         </is>
       </c>
-      <c r="C10" s="10" t="inlineStr"/>
-      <c r="D10" s="9" t="inlineStr">
+      <c r="C12" s="12" t="inlineStr"/>
+      <c r="D12" s="8" t="inlineStr">
         <is>
           <t>°C</t>
         </is>
       </c>
     </row>
-    <row r="11">
-      <c r="A11" s="9" t="inlineStr">
+    <row r="13">
+      <c r="A13" s="8" t="inlineStr">
         <is>
           <t>5a</t>
         </is>
       </c>
-      <c r="B11" s="9" t="inlineStr">
+      <c r="B13" s="8" t="inlineStr">
         <is>
           <t>Licznik dobrych: koniec − początek (naiwnie)</t>
         </is>
       </c>
-      <c r="C11" s="10" t="inlineStr"/>
-      <c r="D11" s="9" t="inlineStr">
+      <c r="C13" s="9" t="inlineStr"/>
+      <c r="D13" s="8" t="inlineStr">
         <is>
           <t>szt.</t>
         </is>
       </c>
     </row>
-    <row r="12">
-      <c r="A12" s="9" t="inlineStr">
+    <row r="14">
+      <c r="A14" s="8" t="inlineStr">
         <is>
           <t>5b</t>
         </is>
       </c>
-      <c r="B12" s="9" t="inlineStr">
+      <c r="B14" s="8" t="inlineStr">
         <is>
           <t>Sztuki dobre w zmianie (suma przyrostów)</t>
         </is>
       </c>
-      <c r="C12" s="10" t="inlineStr"/>
-      <c r="D12" s="9" t="inlineStr">
+      <c r="C14" s="9" t="inlineStr"/>
+      <c r="D14" s="8" t="inlineStr">
         <is>
           <t>szt.</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="9" t="inlineStr">
-        <is>
-          <t>5c</t>
-        </is>
-      </c>
-      <c r="B13" s="9" t="inlineStr">
-        <is>
-          <t>Sztuki złe w zmianie (suma przyrostów)</t>
-        </is>
-      </c>
-      <c r="C13" s="10" t="inlineStr"/>
-      <c r="D13" s="9" t="inlineStr">
-        <is>
-          <t>szt.</t>
-        </is>
-      </c>
-    </row>
-    <row r="14" ht="60" customHeight="1">
-      <c r="A14" s="9" t="inlineStr">
-        <is>
-          <t>6</t>
-        </is>
-      </c>
-      <c r="B14" s="9" t="inlineStr">
-        <is>
-          <t>Ciśnienie: od kiedy do kiedy wartość „zamrożona”? Czy można jej ufać?</t>
-        </is>
-      </c>
-      <c r="C14" s="10" t="inlineStr"/>
-      <c r="D14" s="9" t="inlineStr">
-        <is>
-          <t>opis</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="8" t="inlineStr">
         <is>
+          <t>5c</t>
+        </is>
+      </c>
+      <c r="B15" s="8" t="inlineStr">
+        <is>
+          <t>Sztuki złe w zmianie (suma przyrostów)</t>
+        </is>
+      </c>
+      <c r="C15" s="9" t="inlineStr"/>
+      <c r="D15" s="8" t="inlineStr">
+        <is>
+          <t>szt.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="60" customHeight="1">
+      <c r="A16" s="8" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="B16" s="8" t="inlineStr">
+        <is>
+          <t>Ciśnienie: od kiedy do kiedy wartość „zamrożona”? Czy można jej ufać?</t>
+        </is>
+      </c>
+      <c r="C16" s="11" t="inlineStr"/>
+      <c r="D16" s="8" t="inlineStr">
+        <is>
+          <t>opis</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="5" t="inlineStr">
+        <is>
           <t>Blok 3 — wskaźniki</t>
         </is>
       </c>
     </row>
-    <row r="16">
-      <c r="A16" s="9" t="inlineStr">
+    <row r="18">
+      <c r="A18" s="8" t="inlineStr">
         <is>
           <t>7a</t>
         </is>
       </c>
-      <c r="B16" s="9" t="inlineStr">
+      <c r="B18" s="8" t="inlineStr">
         <is>
           <t>Czas pracy</t>
         </is>
       </c>
-      <c r="C16" s="10" t="inlineStr"/>
-      <c r="D16" s="9" t="inlineStr">
+      <c r="C18" s="12" t="inlineStr"/>
+      <c r="D18" s="8" t="inlineStr">
         <is>
           <t>min</t>
         </is>
       </c>
     </row>
-    <row r="17">
-      <c r="A17" s="9" t="inlineStr">
+    <row r="19">
+      <c r="A19" s="8" t="inlineStr">
         <is>
           <t>7b</t>
         </is>
       </c>
-      <c r="B17" s="9" t="inlineStr">
+      <c r="B19" s="8" t="inlineStr">
         <is>
           <t>Czas postojów (postój + awaria + przezbrojenie)</t>
         </is>
       </c>
-      <c r="C17" s="10" t="inlineStr"/>
-      <c r="D17" s="9" t="inlineStr">
+      <c r="C19" s="12" t="inlineStr"/>
+      <c r="D19" s="8" t="inlineStr">
         <is>
           <t>min</t>
         </is>
       </c>
     </row>
-    <row r="18">
-      <c r="A18" s="9" t="inlineStr">
+    <row r="20">
+      <c r="A20" s="8" t="inlineStr">
         <is>
           <t>8a</t>
         </is>
       </c>
-      <c r="B18" s="9" t="inlineStr">
+      <c r="B20" s="8" t="inlineStr">
         <is>
           <t>Dostępność A</t>
         </is>
       </c>
-      <c r="C18" s="10" t="inlineStr"/>
-      <c r="D18" s="9" t="inlineStr">
+      <c r="C20" s="13" t="inlineStr"/>
+      <c r="D20" s="8" t="inlineStr">
         <is>
           <t>%</t>
         </is>
       </c>
     </row>
-    <row r="19">
-      <c r="A19" s="9" t="inlineStr">
+    <row r="21">
+      <c r="A21" s="8" t="inlineStr">
         <is>
           <t>8b</t>
         </is>
       </c>
-      <c r="B19" s="9" t="inlineStr">
+      <c r="B21" s="8" t="inlineStr">
         <is>
           <t>Wydajność P (cykl idealny 1,5 s = 40 szt./min)</t>
         </is>
       </c>
-      <c r="C19" s="10" t="inlineStr"/>
-      <c r="D19" s="9" t="inlineStr">
+      <c r="C21" s="13" t="inlineStr"/>
+      <c r="D21" s="8" t="inlineStr">
         <is>
           <t>%</t>
         </is>
       </c>
     </row>
-    <row r="20">
-      <c r="A20" s="9" t="inlineStr">
+    <row r="22">
+      <c r="A22" s="8" t="inlineStr">
         <is>
           <t>8c</t>
         </is>
       </c>
-      <c r="B20" s="9" t="inlineStr">
+      <c r="B22" s="8" t="inlineStr">
         <is>
           <t>Jakość Q</t>
         </is>
       </c>
-      <c r="C20" s="10" t="inlineStr"/>
-      <c r="D20" s="9" t="inlineStr">
+      <c r="C22" s="13" t="inlineStr"/>
+      <c r="D22" s="8" t="inlineStr">
         <is>
           <t>%</t>
         </is>
       </c>
     </row>
-    <row r="21">
-      <c r="A21" s="9" t="inlineStr">
+    <row r="23">
+      <c r="A23" s="8" t="inlineStr">
         <is>
           <t>8d</t>
         </is>
       </c>
-      <c r="B21" s="9" t="inlineStr">
+      <c r="B23" s="8" t="inlineStr">
         <is>
           <t>OEE  (zmiana I: 61,7%)</t>
         </is>
       </c>
-      <c r="C21" s="10" t="inlineStr"/>
-      <c r="D21" s="9" t="inlineStr">
+      <c r="C23" s="13" t="inlineStr"/>
+      <c r="D23" s="8" t="inlineStr">
         <is>
           <t>%</t>
         </is>
       </c>
     </row>
-    <row r="22">
-      <c r="A22" s="9" t="inlineStr">
+    <row r="24">
+      <c r="A24" s="8" t="inlineStr">
+        <is>
+          <t>8e</t>
+        </is>
+      </c>
+      <c r="B24" s="8" t="inlineStr">
+        <is>
+          <t>OEE — sprawdzenie: dobre · 1,5 s / 28 800 s</t>
+        </is>
+      </c>
+      <c r="C24" s="13" t="inlineStr"/>
+      <c r="D24" s="8" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="8" t="inlineStr">
         <is>
           <t>9a</t>
         </is>
       </c>
-      <c r="B22" s="9" t="inlineStr">
+      <c r="B25" s="8" t="inlineStr">
         <is>
           <t>Energia zużyta w zmianie</t>
         </is>
       </c>
-      <c r="C22" s="10" t="inlineStr"/>
-      <c r="D22" s="9" t="inlineStr">
+      <c r="C25" s="12" t="inlineStr"/>
+      <c r="D25" s="8" t="inlineStr">
         <is>
           <t>kWh</t>
-        </is>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" s="9" t="inlineStr">
-        <is>
-          <t>9b</t>
-        </is>
-      </c>
-      <c r="B23" s="9" t="inlineStr">
-        <is>
-          <t>Energia na dobrą sztukę  (zmiana I: 8,1 Wh)</t>
-        </is>
-      </c>
-      <c r="C23" s="10" t="inlineStr"/>
-      <c r="D23" s="9" t="inlineStr">
-        <is>
-          <t>Wh/szt.</t>
-        </is>
-      </c>
-    </row>
-    <row r="24" ht="60" customHeight="1">
-      <c r="A24" s="9" t="inlineStr">
-        <is>
-          <t>10a</t>
-        </is>
-      </c>
-      <c r="B24" s="9" t="inlineStr">
-        <is>
-          <t>Pareto — największa przyczyna wg czasu (ile min)</t>
-        </is>
-      </c>
-      <c r="C24" s="10" t="inlineStr"/>
-      <c r="D24" s="9" t="inlineStr">
-        <is>
-          <t>opis</t>
-        </is>
-      </c>
-    </row>
-    <row r="25" ht="60" customHeight="1">
-      <c r="A25" s="9" t="inlineStr">
-        <is>
-          <t>10b</t>
-        </is>
-      </c>
-      <c r="B25" s="9" t="inlineStr">
-        <is>
-          <t>Pareto — największa przyczyna wg liczby zdarzeń (ile)</t>
-        </is>
-      </c>
-      <c r="C25" s="10" t="inlineStr"/>
-      <c r="D25" s="9" t="inlineStr">
-        <is>
-          <t>opis</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="8" t="inlineStr">
         <is>
+          <t>9b</t>
+        </is>
+      </c>
+      <c r="B26" s="8" t="inlineStr">
+        <is>
+          <t>Energia na dobrą sztukę  (zmiana I: 8,1 Wh)</t>
+        </is>
+      </c>
+      <c r="C26" s="14" t="inlineStr"/>
+      <c r="D26" s="8" t="inlineStr">
+        <is>
+          <t>Wh/szt.</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="8" t="inlineStr">
+        <is>
+          <t>9c</t>
+        </is>
+      </c>
+      <c r="B27" s="8" t="inlineStr">
+        <is>
+          <t>Wykonanie planu (plan 14 000 szt.)</t>
+        </is>
+      </c>
+      <c r="C27" s="13" t="inlineStr"/>
+      <c r="D27" s="8" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
+    </row>
+    <row r="28" ht="60" customHeight="1">
+      <c r="A28" s="8" t="inlineStr">
+        <is>
+          <t>10a</t>
+        </is>
+      </c>
+      <c r="B28" s="8" t="inlineStr">
+        <is>
+          <t>Pareto — największa przyczyna wg czasu (ile min)</t>
+        </is>
+      </c>
+      <c r="C28" s="11" t="inlineStr"/>
+      <c r="D28" s="8" t="inlineStr">
+        <is>
+          <t>opis</t>
+        </is>
+      </c>
+    </row>
+    <row r="29" ht="60" customHeight="1">
+      <c r="A29" s="8" t="inlineStr">
+        <is>
+          <t>10b</t>
+        </is>
+      </c>
+      <c r="B29" s="8" t="inlineStr">
+        <is>
+          <t>Pareto — największa przyczyna wg liczby zdarzeń (ile)</t>
+        </is>
+      </c>
+      <c r="C29" s="11" t="inlineStr"/>
+      <c r="D29" s="8" t="inlineStr">
+        <is>
+          <t>opis</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="5" t="inlineStr">
+        <is>
           <t>Blok 4 — karta kontrolna i dashboard</t>
         </is>
       </c>
     </row>
-    <row r="27">
-      <c r="A27" s="9" t="inlineStr">
+    <row r="31">
+      <c r="A31" s="8" t="inlineStr">
         <is>
           <t>11a</t>
         </is>
       </c>
-      <c r="B27" s="9" t="inlineStr">
-        <is>
-          <t>Temperatura: średnia x̄ i odchylenie σ (bez zer)</t>
-        </is>
-      </c>
-      <c r="C27" s="10" t="inlineStr"/>
-      <c r="D27" s="9" t="inlineStr">
+      <c r="B31" s="8" t="inlineStr">
+        <is>
+          <t>Temperatura: średnia x̄ (bez zer)</t>
+        </is>
+      </c>
+      <c r="C31" s="12" t="inlineStr"/>
+      <c r="D31" s="8" t="inlineStr">
         <is>
           <t>°C</t>
         </is>
       </c>
     </row>
-    <row r="28">
-      <c r="A28" s="9" t="inlineStr">
+    <row r="32">
+      <c r="A32" s="8" t="inlineStr">
+        <is>
+          <t>11a</t>
+        </is>
+      </c>
+      <c r="B32" s="8" t="inlineStr">
+        <is>
+          <t>Temperatura: odchylenie standardowe σ (bez zer)</t>
+        </is>
+      </c>
+      <c r="C32" s="12" t="inlineStr"/>
+      <c r="D32" s="8" t="inlineStr">
+        <is>
+          <t>°C</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="8" t="inlineStr">
         <is>
           <t>11b</t>
         </is>
       </c>
-      <c r="B28" s="9" t="inlineStr">
-        <is>
-          <t>Granice kontrolne UCL / LCL</t>
-        </is>
-      </c>
-      <c r="C28" s="10" t="inlineStr"/>
-      <c r="D28" s="9" t="inlineStr">
+      <c r="B33" s="8" t="inlineStr">
+        <is>
+          <t>Górna granica kontrolna UCL</t>
+        </is>
+      </c>
+      <c r="C33" s="12" t="inlineStr"/>
+      <c r="D33" s="8" t="inlineStr">
         <is>
           <t>°C</t>
         </is>
       </c>
     </row>
-    <row r="29">
-      <c r="A29" s="9" t="inlineStr">
+    <row r="34">
+      <c r="A34" s="8" t="inlineStr">
+        <is>
+          <t>11b</t>
+        </is>
+      </c>
+      <c r="B34" s="8" t="inlineStr">
+        <is>
+          <t>Dolna granica kontrolna LCL</t>
+        </is>
+      </c>
+      <c r="C34" s="12" t="inlineStr"/>
+      <c r="D34" s="8" t="inlineStr">
+        <is>
+          <t>°C</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="8" t="inlineStr">
         <is>
           <t>11c</t>
         </is>
       </c>
-      <c r="B29" s="9" t="inlineStr">
-        <is>
-          <t>Kiedy temperatura pierwszy raz przekroczyła UCL? Kiedy była awaria zgrzewu?</t>
-        </is>
-      </c>
-      <c r="C29" s="10" t="inlineStr"/>
-      <c r="D29" s="9" t="inlineStr">
+      <c r="B35" s="8" t="inlineStr">
+        <is>
+          <t>Pierwsze przekroczenie UCL — godzina</t>
+        </is>
+      </c>
+      <c r="C35" s="15" t="inlineStr"/>
+      <c r="D35" s="8" t="inlineStr">
         <is>
           <t>godz.</t>
         </is>
       </c>
     </row>
-    <row r="30">
-      <c r="A30" s="9" t="inlineStr">
+    <row r="36">
+      <c r="A36" s="8" t="inlineStr">
+        <is>
+          <t>11c</t>
+        </is>
+      </c>
+      <c r="B36" s="8" t="inlineStr">
+        <is>
+          <t>Awaria zgrzewu — godzina początku</t>
+        </is>
+      </c>
+      <c r="C36" s="15" t="inlineStr"/>
+      <c r="D36" s="8" t="inlineStr">
+        <is>
+          <t>godz.</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="8" t="inlineStr">
+        <is>
+          <t>11c</t>
+        </is>
+      </c>
+      <c r="B37" s="8" t="inlineStr">
+        <is>
+          <t>Ile minut wcześniej karta dała sygnał?</t>
+        </is>
+      </c>
+      <c r="C37" s="12" t="inlineStr"/>
+      <c r="D37" s="8" t="inlineStr">
+        <is>
+          <t>min</t>
+        </is>
+      </c>
+    </row>
+    <row r="38" ht="60" customHeight="1">
+      <c r="A38" s="8" t="inlineStr">
         <is>
           <t>12</t>
         </is>
       </c>
-      <c r="B30" s="9" t="inlineStr">
-        <is>
-          <t>Dashboard — arkusz „Dashboard” (odbiorca: …………)</t>
-        </is>
-      </c>
-      <c r="C30" s="10" t="inlineStr"/>
-      <c r="D30" s="9" t="inlineStr">
-        <is>
-          <t>arkusz</t>
-        </is>
-      </c>
-    </row>
-    <row r="31" ht="60" customHeight="1">
-      <c r="A31" s="9" t="inlineStr">
+      <c r="B38" s="8" t="inlineStr">
+        <is>
+          <t>Dashboard — arkusz „Dashboard”: dla kogo?</t>
+        </is>
+      </c>
+      <c r="C38" s="11" t="inlineStr"/>
+      <c r="D38" s="8" t="inlineStr">
+        <is>
+          <t>opis</t>
+        </is>
+      </c>
+    </row>
+    <row r="39" ht="60" customHeight="1">
+      <c r="A39" s="8" t="inlineStr">
         <is>
           <t>13</t>
         </is>
       </c>
-      <c r="B31" s="9" t="inlineStr">
+      <c r="B39" s="8" t="inlineStr">
         <is>
           <t>Wnioski dla kierownika: 3 zdania — co poprawić najpierw i dlaczego</t>
         </is>
       </c>
-      <c r="C31" s="10" t="inlineStr"/>
-      <c r="D31" s="9" t="inlineStr">
+      <c r="C39" s="11" t="inlineStr"/>
+      <c r="D39" s="8" t="inlineStr">
         <is>
           <t>opis</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="5">
-    <mergeCell ref="A3:D3"/>
-    <mergeCell ref="A26:D26"/>
-    <mergeCell ref="A15:D15"/>
-    <mergeCell ref="A7:D7"/>
-    <mergeCell ref="B2:D2"/>
+  <mergeCells count="6">
+    <mergeCell ref="A17:D17"/>
+    <mergeCell ref="A8:D8"/>
+    <mergeCell ref="C1:D1"/>
+    <mergeCell ref="A4:D4"/>
+    <mergeCell ref="A30:D30"/>
+    <mergeCell ref="A1:B1"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>